<commit_message>
Integrate all-region PPR atlas and full annual NPP histories
</commit_message>
<xml_diff>
--- a/data/EEZ_008/EEZ_008.xlsx
+++ b/data/EEZ_008/EEZ_008.xlsx
@@ -9,15 +9,18 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Catch" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SPPR" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="sppr_all" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="sppr_inner" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="sppr_PP" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Recycling" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="PPR" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="NPP" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Final mappings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SPPR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="sppr_all" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="sppr_inner" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="sppr_PP" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Recycling" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PPR" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="NPP" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'NPP'!$A$3:$O$73</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -454,13 +457,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1133,6 +1136,9 @@
       <c r="C63" t="n">
         <v>4264873.821</v>
       </c>
+      <c r="D63" t="n">
+        <v>21.4747</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1144,6 +1150,9 @@
       <c r="C64" t="n">
         <v>635027.465</v>
       </c>
+      <c r="D64" t="n">
+        <v>3.5224</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1155,6 +1164,9 @@
       <c r="C65" t="n">
         <v>663483.474</v>
       </c>
+      <c r="D65" t="n">
+        <v>3.6896</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1166,6 +1178,9 @@
       <c r="C66" t="n">
         <v>563239.356</v>
       </c>
+      <c r="D66" t="n">
+        <v>2.9357</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1177,6 +1192,9 @@
       <c r="C67" t="n">
         <v>664386.552</v>
       </c>
+      <c r="D67" t="n">
+        <v>3.6178</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1188,6 +1206,9 @@
       <c r="C68" t="n">
         <v>1463891.629</v>
       </c>
+      <c r="D68" t="n">
+        <v>7.3428</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1199,6 +1220,9 @@
       <c r="C69" t="n">
         <v>1411470.185</v>
       </c>
+      <c r="D69" t="n">
+        <v>6.1923</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1210,6 +1234,9 @@
       <c r="C70" t="n">
         <v>2684460.458</v>
       </c>
+      <c r="D70" t="n">
+        <v>13.6132</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1221,6 +1248,9 @@
       <c r="C71" t="n">
         <v>3248221.422</v>
       </c>
+      <c r="D71" t="n">
+        <v>14.9956</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1232,6 +1262,9 @@
       <c r="C72" t="n">
         <v>1975303.37</v>
       </c>
+      <c r="D72" t="n">
+        <v>9.7636</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1243,6 +1276,9 @@
       <c r="C73" t="n">
         <v>2788837.783</v>
       </c>
+      <c r="D73" t="n">
+        <v>14.2772</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1254,6 +1290,9 @@
       <c r="C74" t="n">
         <v>2467706.614</v>
       </c>
+      <c r="D74" t="n">
+        <v>10.9092</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1265,6 +1304,9 @@
       <c r="C75" t="n">
         <v>3257009.804</v>
       </c>
+      <c r="D75" t="n">
+        <v>13.8167</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1276,6 +1318,9 @@
       <c r="C76" t="n">
         <v>799115.675</v>
       </c>
+      <c r="D76" t="n">
+        <v>4.0121</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1287,6 +1332,9 @@
       <c r="C77" t="n">
         <v>1883325.132</v>
       </c>
+      <c r="D77" t="n">
+        <v>9.0038</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1298,6 +1346,9 @@
       <c r="C78" t="n">
         <v>1961203.295</v>
       </c>
+      <c r="D78" t="n">
+        <v>9.468999999999999</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1309,6 +1360,9 @@
       <c r="C79" t="n">
         <v>1720918.875</v>
       </c>
+      <c r="D79" t="n">
+        <v>8.353899999999999</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1320,6 +1374,9 @@
       <c r="C80" t="n">
         <v>1503226.1</v>
       </c>
+      <c r="D80" t="n">
+        <v>7.192</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1331,6 +1388,9 @@
       <c r="C81" t="n">
         <v>1479663.513</v>
       </c>
+      <c r="D81" t="n">
+        <v>6.8726</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1342,6 +1402,9 @@
       <c r="C82" t="n">
         <v>1500420.777</v>
       </c>
+      <c r="D82" t="n">
+        <v>7.6336</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1353,6 +1416,9 @@
       <c r="C83" t="n">
         <v>1645647.255</v>
       </c>
+      <c r="D83" t="n">
+        <v>7.5063</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1364,22 +1430,2282 @@
       <c r="C84" t="n">
         <v>1553417.155</v>
       </c>
+      <c r="D84" t="n">
+        <v>7.5189</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PPR/NPP converts wet-weight PP to carbon at 9:1; NPP is the fixed 2019 ensemble median.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>PPR/NPP is blank because no NPP estimate exists for this ecosystem.</t>
+          <t>PPR/NPP converts wet-weight PP to carbon at 9:1 and uses the matching year's NPP ensemble median.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>PPR/NPP is blank for years without NPP; see NPP for availability and provenance.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="75" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="65" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Annual net primary production, tonnes carbon per year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PPR/NPP uses the ensemble median for the matching catch year. Blank values are unavailable; no year is substituted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>npp_antoinemorel_tC_yr</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>npp_vgpm_tC_yr</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>npp_eppley_tC_yr</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>npp_cbpm_tC_yr</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>npp_cafe_tC_yr</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>ens_median_tC_yr</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>ens_min_tC_yr</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>ens_max_tC_yr</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>n_models</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>available_models</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>ensemble_basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1950</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1951</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1952</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1953</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1954</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1955</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1956</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1957</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1958</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1959</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1960</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1961</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1962</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1963</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1964</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1965</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1966</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1967</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1968</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1969</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1970</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1971</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1972</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1973</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1974</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1975</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1976</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1977</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1978</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>1979</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>1980</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1981</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>1982</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1983</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>1984</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1985</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>1986</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1987</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1988</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>1990</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1991</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1992</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>1993</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1995</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1996</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1997</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>unsupported</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>reference source has no complete twelve-month year</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B52" t="n">
+        <v>2206670.186959809</v>
+      </c>
+      <c r="G52" t="n">
+        <v>2206670.186959809</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2206670.186959809</v>
+      </c>
+      <c r="I52" t="n">
+        <v>2206670.186959809</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>vgpm: unsupported_year; eppley: unsupported_year; cbpm: unsupported_year; cafe: unsupported_year</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/1998/848d73be4edbdf39/provenance.json</t>
+        </is>
+      </c>
+      <c r="M52" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>antoinemorel</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B53" t="n">
+        <v>2003129.330337425</v>
+      </c>
+      <c r="G53" t="n">
+        <v>2003129.330337425</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2003129.330337425</v>
+      </c>
+      <c r="I53" t="n">
+        <v>2003129.330337425</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>vgpm: unsupported_year; eppley: unsupported_year; cbpm: unsupported_year; cafe: unsupported_year</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/1999/7c2a53b46a02284b/provenance.json</t>
+        </is>
+      </c>
+      <c r="M53" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>antoinemorel</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1998056.744233852</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1998056.744233852</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1998056.744233852</v>
+      </c>
+      <c r="I54" t="n">
+        <v>1998056.744233852</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>vgpm: unsupported_year; eppley: unsupported_year; cbpm: unsupported_year; cafe: unsupported_year</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2000/4061cb7fd4278b03/provenance.json</t>
+        </is>
+      </c>
+      <c r="M54" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>antoinemorel</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B55" t="n">
+        <v>2131783.124165002</v>
+      </c>
+      <c r="G55" t="n">
+        <v>2131783.124165002</v>
+      </c>
+      <c r="H55" t="n">
+        <v>2131783.124165002</v>
+      </c>
+      <c r="I55" t="n">
+        <v>2131783.124165002</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>vgpm: unsupported_year; eppley: unsupported_year; cbpm: unsupported_year; cafe: unsupported_year</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2001/af4237f96f450f68/provenance.json</t>
+        </is>
+      </c>
+      <c r="M55" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>antoinemorel</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2040464.055493773</v>
+      </c>
+      <c r="G56" t="n">
+        <v>2040464.055493773</v>
+      </c>
+      <c r="H56" t="n">
+        <v>2040464.055493773</v>
+      </c>
+      <c r="I56" t="n">
+        <v>2040464.055493773</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>vgpm: unsupported_year; eppley: unsupported_year; cbpm: unsupported_year; cafe: unsupported_year</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2002/cb18d36c3928416f/provenance.json</t>
+        </is>
+      </c>
+      <c r="M56" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>antoinemorel</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B57" t="n">
+        <v>2163551.028815834</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2760858.050486019</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2215163.635700751</v>
+      </c>
+      <c r="E57" t="n">
+        <v>2832971.144091401</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1402904.952613144</v>
+      </c>
+      <c r="G57" t="n">
+        <v>2215163.635700751</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1402904.952613144</v>
+      </c>
+      <c r="I57" t="n">
+        <v>2832971.144091401</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2003/e3b8e4aba049aba8/provenance.json</t>
+        </is>
+      </c>
+      <c r="M57" t="n">
+        <v>5</v>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B58" t="n">
+        <v>2427438.004708632</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3229191.490688191</v>
+      </c>
+      <c r="D58" t="n">
+        <v>2532682.268450878</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3173611.550087711</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1429739.013108294</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2532682.268450878</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1429739.013108294</v>
+      </c>
+      <c r="I58" t="n">
+        <v>3229191.490688191</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2004/1578102eb802e4fd/provenance.json</t>
+        </is>
+      </c>
+      <c r="M58" t="n">
+        <v>5</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B59" t="n">
+        <v>2146017.122047137</v>
+      </c>
+      <c r="C59" t="n">
+        <v>2894348.343489123</v>
+      </c>
+      <c r="D59" t="n">
+        <v>2191057.189137522</v>
+      </c>
+      <c r="E59" t="n">
+        <v>2843540.142234155</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1273924.325318302</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2191057.189137522</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1273924.325318302</v>
+      </c>
+      <c r="I59" t="n">
+        <v>2894348.343489123</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2005/789df515cc84d5eb/provenance.json</t>
+        </is>
+      </c>
+      <c r="M59" t="n">
+        <v>5</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B60" t="n">
+        <v>2364409.917659181</v>
+      </c>
+      <c r="C60" t="n">
+        <v>3118671.338267172</v>
+      </c>
+      <c r="D60" t="n">
+        <v>2406788.656074385</v>
+      </c>
+      <c r="E60" t="n">
+        <v>3199472.92478662</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1382497.929523301</v>
+      </c>
+      <c r="G60" t="n">
+        <v>2406788.656074385</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1382497.929523301</v>
+      </c>
+      <c r="I60" t="n">
+        <v>3199472.92478662</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2006/f986afa7dea50b92/provenance.json</t>
+        </is>
+      </c>
+      <c r="M60" t="n">
+        <v>5</v>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B61" t="n">
+        <v>2247920.675262051</v>
+      </c>
+      <c r="C61" t="n">
+        <v>2829207.645389358</v>
+      </c>
+      <c r="D61" t="n">
+        <v>2205053.108808138</v>
+      </c>
+      <c r="E61" t="n">
+        <v>2949757.309136339</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1268701.209992894</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2247920.675262051</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1268701.209992894</v>
+      </c>
+      <c r="I61" t="n">
+        <v>2949757.309136339</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2007/8f3c65d96b0e1768/provenance.json</t>
+        </is>
+      </c>
+      <c r="M61" t="n">
+        <v>5</v>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B62" t="n">
+        <v>2170396.22760931</v>
+      </c>
+      <c r="C62" t="n">
+        <v>2760509.320839478</v>
+      </c>
+      <c r="D62" t="n">
+        <v>2116435.393800148</v>
+      </c>
+      <c r="E62" t="n">
+        <v>2796721.058940216</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1349281.331216779</v>
+      </c>
+      <c r="G62" t="n">
+        <v>2170396.22760931</v>
+      </c>
+      <c r="H62" t="n">
+        <v>1349281.331216779</v>
+      </c>
+      <c r="I62" t="n">
+        <v>2796721.058940216</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2008/f78aee8d26ee4e4e/provenance.json</t>
+        </is>
+      </c>
+      <c r="M62" t="n">
+        <v>5</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B63" t="n">
+        <v>2421568.480434764</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3101909.441649709</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2513374.174531851</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2959819.662799782</v>
+      </c>
+      <c r="F63" t="n">
+        <v>1431475.269559113</v>
+      </c>
+      <c r="G63" t="n">
+        <v>2513374.174531851</v>
+      </c>
+      <c r="H63" t="n">
+        <v>1431475.269559113</v>
+      </c>
+      <c r="I63" t="n">
+        <v>3101909.441649709</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2009/6fada420a161df7f/provenance.json</t>
+        </is>
+      </c>
+      <c r="M63" t="n">
+        <v>5</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B64" t="n">
+        <v>2467159.936075296</v>
+      </c>
+      <c r="C64" t="n">
+        <v>3391479.617391987</v>
+      </c>
+      <c r="D64" t="n">
+        <v>2619228.488483082</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3031860.87077205</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1446970.036581463</v>
+      </c>
+      <c r="G64" t="n">
+        <v>2619228.488483082</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1446970.036581463</v>
+      </c>
+      <c r="I64" t="n">
+        <v>3391479.617391987</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2010/9faaa1063acdd9a4/provenance.json</t>
+        </is>
+      </c>
+      <c r="M64" t="n">
+        <v>5</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B65" t="n">
+        <v>2206666.031725967</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2741129.34270862</v>
+      </c>
+      <c r="D65" t="n">
+        <v>2213077.947777728</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2954710.358595425</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1334768.754942864</v>
+      </c>
+      <c r="G65" t="n">
+        <v>2213077.947777728</v>
+      </c>
+      <c r="H65" t="n">
+        <v>1334768.754942864</v>
+      </c>
+      <c r="I65" t="n">
+        <v>2954710.358595425</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2011/cda796c56dcdcd17/provenance.json</t>
+        </is>
+      </c>
+      <c r="M65" t="n">
+        <v>5</v>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B66" t="n">
+        <v>2214077.766185705</v>
+      </c>
+      <c r="C66" t="n">
+        <v>2862973.209568417</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2324103.819726762</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2988987.963500179</v>
+      </c>
+      <c r="F66" t="n">
+        <v>1234273.894497019</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2324103.819726762</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1234273.894497019</v>
+      </c>
+      <c r="I66" t="n">
+        <v>2988987.963500179</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2012/c7b676f92b834ce4/provenance.json</t>
+        </is>
+      </c>
+      <c r="M66" t="n">
+        <v>5</v>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B67" t="n">
+        <v>2241438.027956145</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2967425.33644047</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2301307.263169109</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2935215.87879817</v>
+      </c>
+      <c r="F67" t="n">
+        <v>1330839.377377203</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2301307.263169109</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1330839.377377203</v>
+      </c>
+      <c r="I67" t="n">
+        <v>2967425.33644047</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2013/636a6761243c02fa/provenance.json</t>
+        </is>
+      </c>
+      <c r="M67" t="n">
+        <v>5</v>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B68" t="n">
+        <v>2242841.013668565</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2921498.170164058</v>
+      </c>
+      <c r="D68" t="n">
+        <v>2288913.9055572</v>
+      </c>
+      <c r="E68" t="n">
+        <v>3233349.320623446</v>
+      </c>
+      <c r="F68" t="n">
+        <v>1423970.376010197</v>
+      </c>
+      <c r="G68" t="n">
+        <v>2288913.9055572</v>
+      </c>
+      <c r="H68" t="n">
+        <v>1423970.376010197</v>
+      </c>
+      <c r="I68" t="n">
+        <v>3233349.320623446</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2014/f2e604b8075f7f7d/provenance.json</t>
+        </is>
+      </c>
+      <c r="M68" t="n">
+        <v>5</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B69" t="n">
+        <v>2260543.852385257</v>
+      </c>
+      <c r="C69" t="n">
+        <v>2817944.914554722</v>
+      </c>
+      <c r="D69" t="n">
+        <v>2322382.652417133</v>
+      </c>
+      <c r="E69" t="n">
+        <v>2985464.426142581</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1320031.596688144</v>
+      </c>
+      <c r="G69" t="n">
+        <v>2322382.652417133</v>
+      </c>
+      <c r="H69" t="n">
+        <v>1320031.596688144</v>
+      </c>
+      <c r="I69" t="n">
+        <v>2985464.426142581</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2015/f29fd1ff26db87ab/provenance.json</t>
+        </is>
+      </c>
+      <c r="M69" t="n">
+        <v>5</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B70" t="n">
+        <v>2303638.310064568</v>
+      </c>
+      <c r="C70" t="n">
+        <v>3078991.578968809</v>
+      </c>
+      <c r="D70" t="n">
+        <v>2392212.493526156</v>
+      </c>
+      <c r="E70" t="n">
+        <v>3205625.544262341</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1313569.691401121</v>
+      </c>
+      <c r="G70" t="n">
+        <v>2392212.493526156</v>
+      </c>
+      <c r="H70" t="n">
+        <v>1313569.691401121</v>
+      </c>
+      <c r="I70" t="n">
+        <v>3205625.544262341</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2016/66abb99f6b269024/provenance.json</t>
+        </is>
+      </c>
+      <c r="M70" t="n">
+        <v>5</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B71" t="n">
+        <v>2183931.790567559</v>
+      </c>
+      <c r="C71" t="n">
+        <v>2754595.59559341</v>
+      </c>
+      <c r="D71" t="n">
+        <v>2165715.800257812</v>
+      </c>
+      <c r="E71" t="n">
+        <v>3023831.609718118</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1254041.800730962</v>
+      </c>
+      <c r="G71" t="n">
+        <v>2183931.790567559</v>
+      </c>
+      <c r="H71" t="n">
+        <v>1254041.800730962</v>
+      </c>
+      <c r="I71" t="n">
+        <v>3023831.609718118</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2017/9efa693e10f193e3/provenance.json</t>
+        </is>
+      </c>
+      <c r="M71" t="n">
+        <v>5</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B72" t="n">
+        <v>2307797.703692307</v>
+      </c>
+      <c r="C72" t="n">
+        <v>2859837.335787522</v>
+      </c>
+      <c r="D72" t="n">
+        <v>2435934.539857242</v>
+      </c>
+      <c r="E72" t="n">
+        <v>2932968.35201139</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1295749.375662428</v>
+      </c>
+      <c r="G72" t="n">
+        <v>2435934.539857242</v>
+      </c>
+      <c r="H72" t="n">
+        <v>1295749.375662428</v>
+      </c>
+      <c r="I72" t="n">
+        <v>2932968.35201139</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2018/9bc98aadb26d4272/provenance.json</t>
+        </is>
+      </c>
+      <c r="M72" t="n">
+        <v>5</v>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B73" t="n">
+        <v>2188185.406426581</v>
+      </c>
+      <c r="C73" t="n">
+        <v>2860440.329309403</v>
+      </c>
+      <c r="D73" t="n">
+        <v>2295586.311625042</v>
+      </c>
+      <c r="E73" t="n">
+        <v>3207817.38295493</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1243925.771761718</v>
+      </c>
+      <c r="G73" t="n">
+        <v>2295586.311625042</v>
+      </c>
+      <c r="H73" t="n">
+        <v>1243925.771761718</v>
+      </c>
+      <c r="I73" t="n">
+        <v>3207817.38295493</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>NPPExtraction/output/regional_expansion/years/2019/e1437b825b558fb7/provenance.json</t>
+        </is>
+      </c>
+      <c r="M73" t="n">
+        <v>5</v>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>antoinemorel;vgpm;eppley;cbpm;cafe</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>common mask</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:O73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16328,266 +18654,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Specific PPR for EEZ_008</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Simple method, applied per taxon: SPPR = (1/TE)^(TL-1), TE = 0.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>taxon</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>trophic_level</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>sppr_simple</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Dentex dentex</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>4.53</v>
-      </c>
-      <c r="C5" t="n">
-        <v>3388.441561</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Xiphias gladius</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>4.53</v>
-      </c>
-      <c r="C6" t="n">
-        <v>3388.441561</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sarda sarda</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="C7" t="n">
-        <v>3162.27766</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sepia officinalis</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>4.27</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1862.087137</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Auxis rochei</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1348.962883</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Loligo</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>3.99</v>
-      </c>
-      <c r="C10" t="n">
-        <v>977.237221</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Octopus vulgaris</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="C11" t="n">
-        <v>398.107171</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Spicara</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="C12" t="n">
-        <v>380.189396</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Anguilla anguilla</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="C13" t="n">
-        <v>354.813389</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Sardinella aurita</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="C14" t="n">
-        <v>251.188643</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Parapenaeus longirostris</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="C15" t="n">
-        <v>199.526231</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Marine fishes not identified</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="C16" t="n">
-        <v>190.546072</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Engraulis encrasicolus</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3.11</v>
-      </c>
-      <c r="C17" t="n">
-        <v>128.824955</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Sardina pilchardus</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="C18" t="n">
-        <v>114.815362</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Boops boops</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="C19" t="n">
-        <v>61.6595</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Mugilidae</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="C20" t="n">
-        <v>33.884416</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>No Ecopath model has been extracted for this ecosystem yet,</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>so the network-based SPPR methods are not available here.</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No final mappings are available for this ecosystem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Models without a recorded mapping are not assigned invented taxon groups or weights.</t>
         </is>
       </c>
     </row>
@@ -16602,43 +18685,266 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Group SPPR: all</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>All basal sources, including imports. Models are separate. Blank means unavailable, not zero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>group_name</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Specific PPR for EEZ_008</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Simple method, applied per taxon: SPPR = (1/TE)^(TL-1), TE = 0.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>taxon</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>trophic_level</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>sppr_simple</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>No extracted model is available for this ecosystem.</t>
+          <t>Dentex dentex</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3388.441561</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Xiphias gladius</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3388.441561</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sarda sarda</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3162.27766</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sepia officinalis</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1862.087137</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Auxis rochei</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1348.962883</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Loligo</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="C10" t="n">
+        <v>977.237221</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Octopus vulgaris</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>398.107171</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spicara</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="C12" t="n">
+        <v>380.189396</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Anguilla anguilla</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="C13" t="n">
+        <v>354.813389</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sardinella aurita</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C14" t="n">
+        <v>251.188643</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Parapenaeus longirostris</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>199.526231</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Marine fishes not identified</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="C16" t="n">
+        <v>190.546072</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Engraulis encrasicolus</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="C17" t="n">
+        <v>128.824955</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sardina pilchardus</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="C18" t="n">
+        <v>114.815362</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Boops boops</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="C19" t="n">
+        <v>61.6595</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mugilidae</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="C20" t="n">
+        <v>33.884416</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>No Ecopath model has been extracted for this ecosystem yet,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>so the network-based SPPR methods are not available here.</t>
         </is>
       </c>
     </row>
@@ -16663,14 +18969,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Group SPPR: inner</t>
+          <t>Group SPPR: all</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Internal sources: primary producers and detritus; excludes imports. Models are separate. Blank means unavailable, not zero.</t>
+          <t>All basal sources, including imports. Models are separate. Blank means unavailable, not zero.</t>
         </is>
       </c>
     </row>
@@ -16714,14 +19020,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Group SPPR: PP</t>
+          <t>Group SPPR: inner</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Primary producers only; excludes detritus and imports. Models are separate. Blank means unavailable, not zero.</t>
+          <t>Internal sources: primary producers and detritus; excludes imports. Models are separate. Blank means unavailable, not zero.</t>
         </is>
       </c>
     </row>
@@ -16750,6 +19056,57 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Group SPPR: PP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Primary producers only; excludes detritus and imports. Models are separate. Blank means unavailable, not zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>group_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>No extracted model is available for this ecosystem.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16835,7 +19192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20748,32 +23105,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>No net primary production estimate is available for this ecosystem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NPP currently covers LME and High Seas units only, not EEZs.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>